<commit_message>
checking if image upload works when we import file
</commit_message>
<xml_diff>
--- a/frontend/public/product_import_template.xlsx
+++ b/frontend/public/product_import_template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:T2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -512,6 +512,11 @@
           <t>Indicator 6</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Image URL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -596,6 +601,11 @@
       </c>
       <c r="S2" t="n">
         <v>0</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>https://example.com/image.jpg</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>